<commit_message>
Add new bugs to report
</commit_message>
<xml_diff>
--- a/bug-report.xlsx
+++ b/bug-report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maksimsytdikov/Desktop/2gis-qa-task/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F73DCC5-6953-514C-BB5C-F08BB2396EFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AEBDA0F-807B-2C4A-9A1D-6DF9B9EDCB36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="580" yWindow="680" windowWidth="28240" windowHeight="17220" xr2:uid="{73208709-8C2F-2C4C-84FB-0441FB764637}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="32">
   <si>
     <t>Номер</t>
   </si>
@@ -84,10 +84,6 @@
 максимума в 999 символов</t>
   </si>
   <si>
-    <t>POST, /v1/favorites 
-с title &gt; 999</t>
-  </si>
-  <si>
     <t>[API][Favorites] Создание места с сторонними символами</t>
   </si>
   <si>
@@ -100,19 +96,6 @@
   <si>
     <t>POST, /v1/favorites с title = "" 
 или заполненый пробелами</t>
-  </si>
-  <si>
-    <t>[API][Favorites] Создание места с неправильной схемой тела запроса</t>
-  </si>
-  <si>
-    <t>API не валидирует лишние аргументы тела запроса</t>
-  </si>
-  <si>
-    <t>POST, /v1/favorites 
-запрос содержащий в теле любой аргумент не из тз</t>
-  </si>
-  <si>
-    <t>medium</t>
   </si>
   <si>
     <t>[API][Favorites] Неверная время создания места</t>
@@ -135,20 +118,32 @@
 created_at = 15:00 без смещения </t>
   </si>
   <si>
-    <t>lite</t>
-  </si>
-  <si>
-    <t>201 Created, Создано</t>
-  </si>
-  <si>
-    <t>POST, /v1/favorites, с правильным телом запроса</t>
-  </si>
-  <si>
-    <t>При создании места, API возвращает неверный  HTTP статус</t>
-  </si>
-  <si>
-    <t>[API][Favorites] Неверный статус ответа
-создания места</t>
+    <t>[API][Auth] Неверное время жизни токена</t>
+  </si>
+  <si>
+    <t>Жизнь токена состовляет большее кол-во времени чем в тз</t>
+  </si>
+  <si>
+    <t>POST, /v1/favorites, с 
+time.spleep(2.75)</t>
+  </si>
+  <si>
+    <t>401 Unauthorized, 
+«протухший» token</t>
+  </si>
+  <si>
+    <t>POST, /v1/favorites 
+с title = 1000</t>
+  </si>
+  <si>
+    <t>API не валидирует не правильно указанный цвет в теле запроса в нижнем или смешенном регистре</t>
+  </si>
+  <si>
+    <t>POST, /v1/favorites
+c color = "Yellow"</t>
+  </si>
+  <si>
+    <t>[API][Favorites] Создание места с неправильным color</t>
   </si>
 </sst>
 </file>
@@ -578,7 +573,7 @@
         <v>9</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>11</v>
@@ -587,7 +582,7 @@
         <v>8</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
@@ -604,7 +599,7 @@
         <v>14</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>11</v>
@@ -613,7 +608,7 @@
         <v>8</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H3" s="4" t="s">
         <v>10</v>
@@ -624,13 +619,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>11</v>
@@ -639,7 +634,7 @@
         <v>8</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>10</v>
@@ -650,13 +645,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>11</v>
@@ -665,10 +660,10 @@
         <v>8</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="85" x14ac:dyDescent="0.2">
@@ -676,22 +671,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>10</v>
@@ -702,25 +697,25 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>